<commit_message>
Mostra o período filtrado no selo do gráfico
</commit_message>
<xml_diff>
--- a/planilha de gastos.xlsx
+++ b/planilha de gastos.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lorenzo.barcellos\Desktop\lz-analytics\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{01B88450-ABA9-4F45-8C2E-95F98A231F96}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{59D2047B-777D-4A6C-8C02-15559E91E487}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{DCF3DE58-C112-4890-BBC9-14E202ADDC5B}"/>
+    <workbookView xWindow="1320" yWindow="2568" windowWidth="15576" windowHeight="9960" xr2:uid="{DCF3DE58-C112-4890-BBC9-14E202ADDC5B}"/>
   </bookViews>
   <sheets>
     <sheet name="Planilha1" sheetId="1" r:id="rId1"/>

</xml_diff>